<commit_message>
Atualizar checklist com enderecamento IP
</commit_message>
<xml_diff>
--- a/docs/cliente/Checklist_Cliente_Pre_Requisitos_Projeto_Aeroporto.xlsx
+++ b/docs/cliente/Checklist_Cliente_Pre_Requisitos_Projeto_Aeroporto.xlsx
@@ -2,16 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="Rd5e57f1354a84029"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist" sheetId="2" r:id="R9812140aa39b45a0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventario_Ativos" sheetId="3" r:id="R1620f4909a534905"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acessos" sheetId="4" r:id="R545c596b8b794bff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Infraestrutura" sheetId="5" r:id="Red4f2fd3e7334e57"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Portas" sheetId="6" r:id="Rae09570c33144fae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisoes" sheetId="7" r:id="Rc9b79484cacb4c88"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Janelas" sheetId="8" r:id="Rb5e057177252420b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contatos" sheetId="9" r:id="Rb130bb3b65434076"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listas" sheetId="10" r:id="R533f5254d7314704"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="R825f3a99eec84b09"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist" sheetId="2" r:id="R74202503af23459b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventario_Ativos" sheetId="3" r:id="R0931042cc5e14da3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acessos" sheetId="4" r:id="R15935e78068241ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Infraestrutura" sheetId="5" r:id="R76a5d07f34574a83"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enderecamento_IP" sheetId="6" r:id="R1a8197a385d942f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Portas" sheetId="7" r:id="R6c7cb1ca7233409f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisoes" sheetId="8" r:id="R713481524cfa45fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Janelas" sheetId="9" r:id="Rd3caa20d4e9148c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contatos" sheetId="10" r:id="Rc93efc425ba3415a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listas" sheetId="11" r:id="Rc06a584040da4a28"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -172,7 +173,50 @@
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="32">
+  <x:dxfs count="36">
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF006100"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFC6EFCE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF7F6000"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF9C0006"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFF4CCCC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF666666"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFE7E6E6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
     <x:dxf>
       <x:font>
         <x:b/>
@@ -808,7 +852,7 @@
       </x:c>
       <x:c r="B5" s="23" t="n">
         <x:f>COUNTA('Checklist'!A5:A80)</x:f>
-        <x:v>20</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="D5" s="14" t="str">
         <x:v>Inventario validado</x:v>
@@ -852,7 +896,7 @@
       </x:c>
       <x:c r="B7" s="23" t="n">
         <x:f>COUNTIF('Checklist'!H5:H80,"Pendente")</x:f>
-        <x:v>20</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="D7" s="14" t="str">
         <x:v>VMs provisionadas</x:v>
@@ -877,7 +921,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="D8" s="14" t="str">
-        <x:v>Portas liberadas</x:v>
+        <x:v>IPs das VMs e VIPs definidos</x:v>
       </x:c>
       <x:c r="E8" s="25" t="n">
         <x:v>46246</x:v>
@@ -887,7 +931,7 @@
       </x:c>
       <x:c r="G8" s="14" t="str"/>
       <x:c r="H8" s="14" t="str">
-        <x:v>SNMP, ICMP, SSH/Telnet, HTTPS e comunicacao interna</x:v>
+        <x:v>Obrigatorio para provisionamento e DNS</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="31.5" hidden="0" customHeight="1">
@@ -899,17 +943,17 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="D9" s="14" t="str">
-        <x:v>Janelas aprovadas</x:v>
+        <x:v>Portas liberadas</x:v>
       </x:c>
       <x:c r="E9" s="25" t="n">
-        <x:v>46247</x:v>
+        <x:v>46246</x:v>
       </x:c>
       <x:c r="F9" s="14" t="str">
         <x:v>Pendente</x:v>
       </x:c>
       <x:c r="G9" s="14" t="str"/>
       <x:c r="H9" s="14" t="str">
-        <x:v>Failover, backup/restore e rede</x:v>
+        <x:v>SNMP, ICMP, SSH/Telnet, HTTPS e comunicacao interna</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="31.5" hidden="0" customHeight="1">
@@ -921,26 +965,39 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="D10" s="14" t="str">
-        <x:v>Kickoff autorizado</x:v>
+        <x:v>Janelas aprovadas</x:v>
       </x:c>
       <x:c r="E10" s="25" t="n">
-        <x:v>46249</x:v>
+        <x:v>46247</x:v>
       </x:c>
       <x:c r="F10" s="14" t="str">
         <x:v>Pendente</x:v>
       </x:c>
       <x:c r="G10" s="14" t="str"/>
       <x:c r="H10" s="14" t="str">
-        <x:v>Inicio planejado do projeto</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="15" hidden="0" customHeight="1">
+        <x:v>Failover, backup/restore e rede</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="31.5" hidden="0" customHeight="1">
       <x:c r="A11" s="14" t="str">
         <x:v>Bloqueadores de alta prioridade</x:v>
       </x:c>
       <x:c r="B11" s="23" t="n">
         <x:f>COUNTIFS('Checklist'!G5:G80,"Alta",'Checklist'!H5:H80,"Pendente")</x:f>
-        <x:v>13</x:v>
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="D11" t="str">
+        <x:v>Kickoff autorizado</x:v>
+      </x:c>
+      <x:c r="E11" s="26" t="n">
+        <x:v>46249</x:v>
+      </x:c>
+      <x:c r="F11" t="str">
+        <x:v>Pendente</x:v>
+      </x:c>
+      <x:c r="G11" t="str"/>
+      <x:c r="H11" t="str">
+        <x:v>Inicio planejado do projeto</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -948,14 +1005,14 @@
     <x:mergeCell ref="A1:H1"/>
     <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="F5:F10">
+  <x:conditionalFormatting sqref="F5:F11">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Concluido"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Em andamento"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Pendente"/>
     <x:cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="Nao aplicavel"/>
   </x:conditionalFormatting>
   <x:dataValidations count="1">
-    <x:dataValidation type="list" sqref="F5:F10">
+    <x:dataValidation type="list" sqref="F5:F11">
       <x:formula1>"Pendente,Em andamento,Concluido,Nao aplicavel"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -964,6 +1021,206 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="52.380001068115234" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="52.380001068115234" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="52.380001068115234" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="52.380001068115234" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="52.380001068115234" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="31.25" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="31.25" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="31.25" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="19.200000762939453" hidden="0" customHeight="1">
+      <x:c r="A1" s="6" t="str">
+        <x:v>Contatos e Responsaveis</x:v>
+      </x:c>
+      <x:c r="B1" s="6" t="str">
+        <x:v>Contatos e Responsaveis</x:v>
+      </x:c>
+      <x:c r="C1" s="6" t="str">
+        <x:v>Contatos e Responsaveis</x:v>
+      </x:c>
+      <x:c r="D1" s="6" t="str">
+        <x:v>Contatos e Responsaveis</x:v>
+      </x:c>
+      <x:c r="E1" s="6" t="str">
+        <x:v>Contatos e Responsaveis</x:v>
+      </x:c>
+      <x:c r="F1" s="6" t="str">
+        <x:v>Contatos e Responsaveis</x:v>
+      </x:c>
+      <x:c r="G1" s="6" t="str">
+        <x:v>Contatos e Responsaveis</x:v>
+      </x:c>
+      <x:c r="H1" s="6" t="str">
+        <x:v>Contatos e Responsaveis</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2" s="11" t="str">
+        <x:v>Preencher responsaveis por area para aprovacoes, duvidas e escalonamento.</x:v>
+      </x:c>
+      <x:c r="B2" s="11" t="str">
+        <x:v>Preencher responsaveis por area para aprovacoes, duvidas e escalonamento.</x:v>
+      </x:c>
+      <x:c r="C2" s="11" t="str">
+        <x:v>Preencher responsaveis por area para aprovacoes, duvidas e escalonamento.</x:v>
+      </x:c>
+      <x:c r="D2" s="11" t="str">
+        <x:v>Preencher responsaveis por area para aprovacoes, duvidas e escalonamento.</x:v>
+      </x:c>
+      <x:c r="E2" s="11" t="str">
+        <x:v>Preencher responsaveis por area para aprovacoes, duvidas e escalonamento.</x:v>
+      </x:c>
+      <x:c r="F2" s="11" t="str">
+        <x:v>Preencher responsaveis por area para aprovacoes, duvidas e escalonamento.</x:v>
+      </x:c>
+      <x:c r="G2" s="11" t="str">
+        <x:v>Preencher responsaveis por area para aprovacoes, duvidas e escalonamento.</x:v>
+      </x:c>
+      <x:c r="H2" s="11" t="str">
+        <x:v>Preencher responsaveis por area para aprovacoes, duvidas e escalonamento.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3"/>
+    <x:row r="4" ht="15" hidden="0" customHeight="1">
+      <x:c r="A4" s="17" t="str">
+        <x:v>Area</x:v>
+      </x:c>
+      <x:c r="B4" s="17" t="str">
+        <x:v>Nome</x:v>
+      </x:c>
+      <x:c r="C4" s="17" t="str">
+        <x:v>Cargo/Funcao</x:v>
+      </x:c>
+      <x:c r="D4" s="17" t="str">
+        <x:v>E-mail</x:v>
+      </x:c>
+      <x:c r="E4" s="17" t="str">
+        <x:v>Telefone</x:v>
+      </x:c>
+      <x:c r="F4" s="17" t="str">
+        <x:v>Responsabilidade</x:v>
+      </x:c>
+      <x:c r="G4" s="17" t="str">
+        <x:v>Backup</x:v>
+      </x:c>
+      <x:c r="H4" s="17" t="str">
+        <x:v>Observacoes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="15" hidden="0" customHeight="1">
+      <x:c r="A5" s="14" t="str">
+        <x:v>Gestao do projeto</x:v>
+      </x:c>
+      <x:c r="B5" s="14" t="str"/>
+      <x:c r="C5" s="14" t="str"/>
+      <x:c r="D5" s="14" t="str"/>
+      <x:c r="E5" s="14" t="str"/>
+      <x:c r="F5" s="14" t="str">
+        <x:v>Aprovacao de cronograma e status report</x:v>
+      </x:c>
+      <x:c r="G5" s="14" t="str"/>
+      <x:c r="H5" s="14" t="str"/>
+    </x:row>
+    <x:row r="6" ht="15" hidden="0" customHeight="1">
+      <x:c r="A6" s="14" t="str">
+        <x:v>Rede</x:v>
+      </x:c>
+      <x:c r="B6" s="14" t="str"/>
+      <x:c r="C6" s="14" t="str"/>
+      <x:c r="D6" s="14" t="str"/>
+      <x:c r="E6" s="14" t="str"/>
+      <x:c r="F6" s="14" t="str">
+        <x:v>Portas, VLANs, ACLs, QoS e roteamento</x:v>
+      </x:c>
+      <x:c r="G6" s="14" t="str"/>
+      <x:c r="H6" s="14" t="str"/>
+    </x:row>
+    <x:row r="7" ht="15" hidden="0" customHeight="1">
+      <x:c r="A7" s="14" t="str">
+        <x:v>Seguranca</x:v>
+      </x:c>
+      <x:c r="B7" s="14" t="str"/>
+      <x:c r="C7" s="14" t="str"/>
+      <x:c r="D7" s="14" t="str"/>
+      <x:c r="E7" s="14" t="str"/>
+      <x:c r="F7" s="14" t="str">
+        <x:v>VPN, credenciais, certificados e RBAC</x:v>
+      </x:c>
+      <x:c r="G7" s="14" t="str"/>
+      <x:c r="H7" s="14" t="str"/>
+    </x:row>
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
+      <x:c r="A8" s="14" t="str">
+        <x:v>Infraestrutura</x:v>
+      </x:c>
+      <x:c r="B8" s="14" t="str"/>
+      <x:c r="C8" s="14" t="str"/>
+      <x:c r="D8" s="14" t="str"/>
+      <x:c r="E8" s="14" t="str"/>
+      <x:c r="F8" s="14" t="str">
+        <x:v>VMs, storage, DNS, NTP e SO</x:v>
+      </x:c>
+      <x:c r="G8" s="14" t="str"/>
+      <x:c r="H8" s="14" t="str"/>
+    </x:row>
+    <x:row r="9" ht="15" hidden="0" customHeight="1">
+      <x:c r="A9" s="14" t="str">
+        <x:v>Banco de dados</x:v>
+      </x:c>
+      <x:c r="B9" s="14" t="str"/>
+      <x:c r="C9" s="14" t="str"/>
+      <x:c r="D9" s="14" t="str"/>
+      <x:c r="E9" s="14" t="str"/>
+      <x:c r="F9" s="14" t="str">
+        <x:v>PostgreSQL, backup, restore e performance</x:v>
+      </x:c>
+      <x:c r="G9" s="14" t="str"/>
+      <x:c r="H9" s="14" t="str"/>
+    </x:row>
+    <x:row r="10" ht="15" hidden="0" customHeight="1">
+      <x:c r="A10" s="14" t="str">
+        <x:v>Operacao/NOC</x:v>
+      </x:c>
+      <x:c r="B10" s="14" t="str"/>
+      <x:c r="C10" s="14" t="str"/>
+      <x:c r="D10" s="14" t="str"/>
+      <x:c r="E10" s="14" t="str"/>
+      <x:c r="F10" s="14" t="str">
+        <x:v>Recebimento de alertas e operacao assistida</x:v>
+      </x:c>
+      <x:c r="G10" s="14" t="str"/>
+      <x:c r="H10" s="14" t="str"/>
+    </x:row>
+    <x:row r="11" ht="15" hidden="0" customHeight="1">
+      <x:c r="A11" s="14" t="str">
+        <x:v>Aplicacoes</x:v>
+      </x:c>
+      <x:c r="B11" s="14" t="str"/>
+      <x:c r="C11" s="14" t="str"/>
+      <x:c r="D11" s="14" t="str"/>
+      <x:c r="E11" s="14" t="str"/>
+      <x:c r="F11" s="14" t="str">
+        <x:v>Validacao de servicos monitorados</x:v>
+      </x:c>
+      <x:c r="G11" s="14" t="str"/>
+      <x:c r="H11" s="14" t="str"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:H1"/>
+    <x:mergeCell ref="A2:H2"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -1418,13 +1675,13 @@
         <x:v>Infraestrutura</x:v>
       </x:c>
       <x:c r="C13" s="14" t="str">
-        <x:v>Storage NVMe para PostgreSQL</x:v>
+        <x:v>Enderecamento IP das VMs</x:v>
       </x:c>
       <x:c r="D13" s="14" t="str">
-        <x:v>Obrigatorio para banco com retencao de 180 dias.</x:v>
+        <x:v>Definir IP, mascara, gateway, VLAN/sub-rede e DNS de cada VM.</x:v>
       </x:c>
       <x:c r="E13" s="14" t="str">
-        <x:v>Evidencia tecnica</x:v>
+        <x:v>Aba Enderecamento_IP</x:v>
       </x:c>
       <x:c r="F13" s="14" t="str"/>
       <x:c r="G13" s="14" t="str">
@@ -1443,13 +1700,13 @@
         <x:v>Infraestrutura</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>DNS e NTP</x:v>
+        <x:v>VIPs da solucao</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
-        <x:v>Resolucao de nomes e sincronismo de horario.</x:v>
+        <x:v>Definir VIPs para acesso web/HA e nomes DNS associados.</x:v>
       </x:c>
       <x:c r="E14" s="14" t="str">
-        <x:v>Configuracao validada</x:v>
+        <x:v>Aba Enderecamento_IP</x:v>
       </x:c>
       <x:c r="F14" s="14" t="str"/>
       <x:c r="G14" s="14" t="str">
@@ -1465,20 +1722,20 @@
         <x:v>CLI-011</x:v>
       </x:c>
       <x:c r="B15" s="14" t="str">
-        <x:v>Rede</x:v>
+        <x:v>Infraestrutura</x:v>
       </x:c>
       <x:c r="C15" s="14" t="str">
-        <x:v>VLAN de monitoramento</x:v>
+        <x:v>Storage NVMe para PostgreSQL</x:v>
       </x:c>
       <x:c r="D15" s="14" t="str">
-        <x:v>Recomendada para trafego da solucao.</x:v>
+        <x:v>Obrigatorio para banco com retencao de 180 dias.</x:v>
       </x:c>
       <x:c r="E15" s="14" t="str">
-        <x:v>Desenho/rede</x:v>
+        <x:v>Evidencia tecnica</x:v>
       </x:c>
       <x:c r="F15" s="14" t="str"/>
       <x:c r="G15" s="14" t="str">
-        <x:v>Media</x:v>
+        <x:v>Alta</x:v>
       </x:c>
       <x:c r="H15" s="14" t="str">
         <x:v>Pendente</x:v>
@@ -1490,16 +1747,16 @@
         <x:v>CLI-012</x:v>
       </x:c>
       <x:c r="B16" s="14" t="str">
-        <x:v>Rede</x:v>
+        <x:v>Infraestrutura</x:v>
       </x:c>
       <x:c r="C16" s="14" t="str">
-        <x:v>Liberacao de portas</x:v>
+        <x:v>DNS e NTP</x:v>
       </x:c>
       <x:c r="D16" s="14" t="str">
-        <x:v>SNMP, ICMP, SSH/Telnet, HTTPS e comunicacoes internas.</x:v>
+        <x:v>Resolucao de nomes e sincronismo de horario.</x:v>
       </x:c>
       <x:c r="E16" s="14" t="str">
-        <x:v>Matriz de firewall</x:v>
+        <x:v>Configuracao validada</x:v>
       </x:c>
       <x:c r="F16" s="14" t="str"/>
       <x:c r="G16" s="14" t="str">
@@ -1515,16 +1772,16 @@
         <x:v>CLI-013</x:v>
       </x:c>
       <x:c r="B17" s="14" t="str">
-        <x:v>Seguranca</x:v>
+        <x:v>Rede</x:v>
       </x:c>
       <x:c r="C17" s="14" t="str">
-        <x:v>Certificados TLS/HTTPS</x:v>
+        <x:v>VLAN de monitoramento</x:v>
       </x:c>
       <x:c r="D17" s="14" t="str">
-        <x:v>Certificados para frontend, Grafana, AWX e VIP quando aplicavel.</x:v>
+        <x:v>Recomendada para trafego da solucao.</x:v>
       </x:c>
       <x:c r="E17" s="14" t="str">
-        <x:v>Certificados</x:v>
+        <x:v>Desenho/rede</x:v>
       </x:c>
       <x:c r="F17" s="14" t="str"/>
       <x:c r="G17" s="14" t="str">
@@ -1540,16 +1797,16 @@
         <x:v>CLI-014</x:v>
       </x:c>
       <x:c r="B18" s="14" t="str">
-        <x:v>Decisoes</x:v>
+        <x:v>Rede</x:v>
       </x:c>
       <x:c r="C18" s="14" t="str">
-        <x:v>Retencao de dados</x:v>
+        <x:v>Liberacao de portas</x:v>
       </x:c>
       <x:c r="D18" s="14" t="str">
-        <x:v>Confirmar politica de 180 dias.</x:v>
+        <x:v>SNMP, ICMP, SSH/Telnet, HTTPS e comunicacoes internas.</x:v>
       </x:c>
       <x:c r="E18" s="14" t="str">
-        <x:v>Aprovacao formal</x:v>
+        <x:v>Matriz de firewall</x:v>
       </x:c>
       <x:c r="F18" s="14" t="str"/>
       <x:c r="G18" s="14" t="str">
@@ -1565,16 +1822,16 @@
         <x:v>CLI-015</x:v>
       </x:c>
       <x:c r="B19" s="14" t="str">
-        <x:v>Decisoes</x:v>
+        <x:v>Seguranca</x:v>
       </x:c>
       <x:c r="C19" s="14" t="str">
-        <x:v>AWX standby</x:v>
+        <x:v>Certificados TLS/HTTPS</x:v>
       </x:c>
       <x:c r="D19" s="14" t="str">
-        <x:v>Definir se standby sera obrigatorio ou opcional no aceite.</x:v>
+        <x:v>Certificados para frontend, Grafana, AWX e VIP quando aplicavel.</x:v>
       </x:c>
       <x:c r="E19" s="14" t="str">
-        <x:v>Decisao formal</x:v>
+        <x:v>Certificados</x:v>
       </x:c>
       <x:c r="F19" s="14" t="str"/>
       <x:c r="G19" s="14" t="str">
@@ -1590,16 +1847,16 @@
         <x:v>CLI-016</x:v>
       </x:c>
       <x:c r="B20" s="14" t="str">
-        <x:v>Operacao</x:v>
+        <x:v>Decisoes</x:v>
       </x:c>
       <x:c r="C20" s="14" t="str">
-        <x:v>Contatos de escalonamento</x:v>
+        <x:v>Retencao de dados</x:v>
       </x:c>
       <x:c r="D20" s="14" t="str">
-        <x:v>Responsaveis por rede, infra, banco, seguranca e operacao.</x:v>
+        <x:v>Confirmar politica de 180 dias.</x:v>
       </x:c>
       <x:c r="E20" s="14" t="str">
-        <x:v>Planilha</x:v>
+        <x:v>Aprovacao formal</x:v>
       </x:c>
       <x:c r="F20" s="14" t="str"/>
       <x:c r="G20" s="14" t="str">
@@ -1615,20 +1872,20 @@
         <x:v>CLI-017</x:v>
       </x:c>
       <x:c r="B21" s="14" t="str">
-        <x:v>Operacao</x:v>
+        <x:v>Decisoes</x:v>
       </x:c>
       <x:c r="C21" s="14" t="str">
-        <x:v>Janelas de mudanca</x:v>
+        <x:v>AWX standby</x:v>
       </x:c>
       <x:c r="D21" s="14" t="str">
-        <x:v>Instalacao, failover, backup/restore, VLANs, ACLs e QoS.</x:v>
+        <x:v>Definir se standby sera obrigatorio ou opcional no aceite.</x:v>
       </x:c>
       <x:c r="E21" s="14" t="str">
-        <x:v>Calendario aprovado</x:v>
+        <x:v>Decisao formal</x:v>
       </x:c>
       <x:c r="F21" s="14" t="str"/>
       <x:c r="G21" s="14" t="str">
-        <x:v>Alta</x:v>
+        <x:v>Media</x:v>
       </x:c>
       <x:c r="H21" s="14" t="str">
         <x:v>Pendente</x:v>
@@ -1643,17 +1900,17 @@
         <x:v>Operacao</x:v>
       </x:c>
       <x:c r="C22" s="14" t="str">
-        <x:v>Modelo de relatorio</x:v>
+        <x:v>Contatos de escalonamento</x:v>
       </x:c>
       <x:c r="D22" s="14" t="str">
-        <x:v>Expectativa de relatorios executivos e CSV/Excel.</x:v>
+        <x:v>Responsaveis por rede, infra, banco, seguranca e operacao.</x:v>
       </x:c>
       <x:c r="E22" s="14" t="str">
-        <x:v>Modelo/exemplo</x:v>
+        <x:v>Planilha</x:v>
       </x:c>
       <x:c r="F22" s="14" t="str"/>
       <x:c r="G22" s="14" t="str">
-        <x:v>Baixa</x:v>
+        <x:v>Alta</x:v>
       </x:c>
       <x:c r="H22" s="14" t="str">
         <x:v>Pendente</x:v>
@@ -1668,17 +1925,17 @@
         <x:v>Operacao</x:v>
       </x:c>
       <x:c r="C23" s="14" t="str">
-        <x:v>Publico do treinamento</x:v>
+        <x:v>Janelas de mudanca</x:v>
       </x:c>
       <x:c r="D23" s="14" t="str">
-        <x:v>Lista de participantes e perfis.</x:v>
+        <x:v>Instalacao, failover, backup/restore, VLANs, ACLs e QoS.</x:v>
       </x:c>
       <x:c r="E23" s="14" t="str">
-        <x:v>Lista</x:v>
+        <x:v>Calendario aprovado</x:v>
       </x:c>
       <x:c r="F23" s="14" t="str"/>
       <x:c r="G23" s="14" t="str">
-        <x:v>Media</x:v>
+        <x:v>Alta</x:v>
       </x:c>
       <x:c r="H23" s="14" t="str">
         <x:v>Pendente</x:v>
@@ -1690,25 +1947,75 @@
         <x:v>CLI-020</x:v>
       </x:c>
       <x:c r="B24" s="14" t="str">
-        <x:v>Aceite</x:v>
+        <x:v>Operacao</x:v>
       </x:c>
       <x:c r="C24" s="14" t="str">
-        <x:v>Aprovadores do projeto</x:v>
+        <x:v>Modelo de relatorio</x:v>
       </x:c>
       <x:c r="D24" s="14" t="str">
-        <x:v>Quem aprova arquitetura, piloto, ondas, restore e aceite final.</x:v>
+        <x:v>Expectativa de relatorios executivos e CSV/Excel.</x:v>
       </x:c>
       <x:c r="E24" s="14" t="str">
-        <x:v>Lista</x:v>
+        <x:v>Modelo/exemplo</x:v>
       </x:c>
       <x:c r="F24" s="14" t="str"/>
       <x:c r="G24" s="14" t="str">
+        <x:v>Baixa</x:v>
+      </x:c>
+      <x:c r="H24" s="14" t="str">
+        <x:v>Pendente</x:v>
+      </x:c>
+      <x:c r="I24" s="14" t="str"/>
+    </x:row>
+    <x:row r="25" ht="15" hidden="0" customHeight="1">
+      <x:c r="A25" s="14" t="str">
+        <x:v>CLI-021</x:v>
+      </x:c>
+      <x:c r="B25" s="14" t="str">
+        <x:v>Operacao</x:v>
+      </x:c>
+      <x:c r="C25" s="14" t="str">
+        <x:v>Publico do treinamento</x:v>
+      </x:c>
+      <x:c r="D25" s="14" t="str">
+        <x:v>Lista de participantes e perfis.</x:v>
+      </x:c>
+      <x:c r="E25" s="14" t="str">
+        <x:v>Lista</x:v>
+      </x:c>
+      <x:c r="F25" s="14" t="str"/>
+      <x:c r="G25" s="14" t="str">
+        <x:v>Media</x:v>
+      </x:c>
+      <x:c r="H25" s="14" t="str">
+        <x:v>Pendente</x:v>
+      </x:c>
+      <x:c r="I25" s="14" t="str"/>
+    </x:row>
+    <x:row r="26" ht="15" hidden="0" customHeight="1">
+      <x:c r="A26" s="14" t="str">
+        <x:v>CLI-022</x:v>
+      </x:c>
+      <x:c r="B26" s="14" t="str">
+        <x:v>Aceite</x:v>
+      </x:c>
+      <x:c r="C26" s="14" t="str">
+        <x:v>Aprovadores do projeto</x:v>
+      </x:c>
+      <x:c r="D26" s="14" t="str">
+        <x:v>Quem aprova arquitetura, piloto, ondas, restore e aceite final.</x:v>
+      </x:c>
+      <x:c r="E26" s="14" t="str">
+        <x:v>Lista</x:v>
+      </x:c>
+      <x:c r="F26" s="14" t="str"/>
+      <x:c r="G26" s="14" t="str">
         <x:v>Alta</x:v>
       </x:c>
-      <x:c r="H24" s="14" t="str">
-        <x:v>Pendente</x:v>
-      </x:c>
-      <x:c r="I24" s="14" t="str"/>
+      <x:c r="H26" s="14" t="str">
+        <x:v>Pendente</x:v>
+      </x:c>
+      <x:c r="I26" s="14" t="str"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -16946,6 +17253,574 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
+    <x:col min="1" max="1" width="10" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="23.75" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="23.75" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="88.12999725341797" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18.75" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="18.75" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="18.75" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="18.75" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="18.75" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="38" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="38" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="38" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="35" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="19.200000762939453" hidden="0" customHeight="1">
+      <x:c r="A1" s="6" t="str">
+        <x:v>Enderecamento IP das VMs e VIPs</x:v>
+      </x:c>
+      <x:c r="B1" s="6" t="str">
+        <x:v>Enderecamento IP das VMs e VIPs</x:v>
+      </x:c>
+      <x:c r="C1" s="6" t="str">
+        <x:v>Enderecamento IP das VMs e VIPs</x:v>
+      </x:c>
+      <x:c r="D1" s="6" t="str">
+        <x:v>Enderecamento IP das VMs e VIPs</x:v>
+      </x:c>
+      <x:c r="E1" s="6" t="str">
+        <x:v>Enderecamento IP das VMs e VIPs</x:v>
+      </x:c>
+      <x:c r="F1" s="6" t="str">
+        <x:v>Enderecamento IP das VMs e VIPs</x:v>
+      </x:c>
+      <x:c r="G1" s="6" t="str">
+        <x:v>Enderecamento IP das VMs e VIPs</x:v>
+      </x:c>
+      <x:c r="H1" s="6" t="str">
+        <x:v>Enderecamento IP das VMs e VIPs</x:v>
+      </x:c>
+      <x:c r="I1" s="6" t="str">
+        <x:v>Enderecamento IP das VMs e VIPs</x:v>
+      </x:c>
+      <x:c r="J1" s="6" t="str">
+        <x:v>Enderecamento IP das VMs e VIPs</x:v>
+      </x:c>
+      <x:c r="K1" s="6" t="str">
+        <x:v>Enderecamento IP das VMs e VIPs</x:v>
+      </x:c>
+      <x:c r="L1" s="6" t="str">
+        <x:v>Enderecamento IP das VMs e VIPs</x:v>
+      </x:c>
+      <x:c r="M1" s="6" t="str">
+        <x:v>Enderecamento IP das VMs e VIPs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2" s="11" t="str">
+        <x:v>O cliente deve definir ou disponibilizar os IPs, sub-redes, gateways, VLANs e nomes DNS antes do provisionamento e da instalacao.</x:v>
+      </x:c>
+      <x:c r="B2" s="11" t="str">
+        <x:v>O cliente deve definir ou disponibilizar os IPs, sub-redes, gateways, VLANs e nomes DNS antes do provisionamento e da instalacao.</x:v>
+      </x:c>
+      <x:c r="C2" s="11" t="str">
+        <x:v>O cliente deve definir ou disponibilizar os IPs, sub-redes, gateways, VLANs e nomes DNS antes do provisionamento e da instalacao.</x:v>
+      </x:c>
+      <x:c r="D2" s="11" t="str">
+        <x:v>O cliente deve definir ou disponibilizar os IPs, sub-redes, gateways, VLANs e nomes DNS antes do provisionamento e da instalacao.</x:v>
+      </x:c>
+      <x:c r="E2" s="11" t="str">
+        <x:v>O cliente deve definir ou disponibilizar os IPs, sub-redes, gateways, VLANs e nomes DNS antes do provisionamento e da instalacao.</x:v>
+      </x:c>
+      <x:c r="F2" s="11" t="str">
+        <x:v>O cliente deve definir ou disponibilizar os IPs, sub-redes, gateways, VLANs e nomes DNS antes do provisionamento e da instalacao.</x:v>
+      </x:c>
+      <x:c r="G2" s="11" t="str">
+        <x:v>O cliente deve definir ou disponibilizar os IPs, sub-redes, gateways, VLANs e nomes DNS antes do provisionamento e da instalacao.</x:v>
+      </x:c>
+      <x:c r="H2" s="11" t="str">
+        <x:v>O cliente deve definir ou disponibilizar os IPs, sub-redes, gateways, VLANs e nomes DNS antes do provisionamento e da instalacao.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3"/>
+    <x:row r="4" ht="15" hidden="0" customHeight="1">
+      <x:c r="A4" s="17" t="str">
+        <x:v>ID</x:v>
+      </x:c>
+      <x:c r="B4" s="17" t="str">
+        <x:v>Componente</x:v>
+      </x:c>
+      <x:c r="C4" s="17" t="str">
+        <x:v>Funcao</x:v>
+      </x:c>
+      <x:c r="D4" s="17" t="str">
+        <x:v>Ambiente</x:v>
+      </x:c>
+      <x:c r="E4" s="17" t="str">
+        <x:v>IP definido</x:v>
+      </x:c>
+      <x:c r="F4" s="17" t="str">
+        <x:v>Mascara/CIDR</x:v>
+      </x:c>
+      <x:c r="G4" s="17" t="str">
+        <x:v>Gateway</x:v>
+      </x:c>
+      <x:c r="H4" s="17" t="str">
+        <x:v>VLAN/Sub-rede</x:v>
+      </x:c>
+      <x:c r="I4" s="17" t="str">
+        <x:v>DNS/FQDN</x:v>
+      </x:c>
+      <x:c r="J4" s="17" t="str">
+        <x:v>NAT/Publicacao</x:v>
+      </x:c>
+      <x:c r="K4" s="17" t="str">
+        <x:v>Responsavel cliente</x:v>
+      </x:c>
+      <x:c r="L4" s="17" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+      <x:c r="M4" s="17" t="str">
+        <x:v>Observacoes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="15" hidden="0" customHeight="1">
+      <x:c r="A5" s="14" t="str">
+        <x:v>IP-001</x:v>
+      </x:c>
+      <x:c r="B5" s="14" t="str">
+        <x:v>zbx-server-01</x:v>
+      </x:c>
+      <x:c r="C5" s="14" t="str">
+        <x:v>Zabbix Server ativo</x:v>
+      </x:c>
+      <x:c r="D5" s="14" t="str">
+        <x:v>Producao</x:v>
+      </x:c>
+      <x:c r="E5" s="14" t="str"/>
+      <x:c r="F5" s="14" t="str"/>
+      <x:c r="G5" s="14" t="str"/>
+      <x:c r="H5" s="14" t="str"/>
+      <x:c r="I5" s="14" t="str"/>
+      <x:c r="J5" s="14" t="str">
+        <x:v>Nao</x:v>
+      </x:c>
+      <x:c r="K5" s="14" t="str"/>
+      <x:c r="L5" s="14" t="str">
+        <x:v>Pendente</x:v>
+      </x:c>
+      <x:c r="M5" s="14" t="str"/>
+    </x:row>
+    <x:row r="6" ht="15" hidden="0" customHeight="1">
+      <x:c r="A6" s="14" t="str">
+        <x:v>IP-002</x:v>
+      </x:c>
+      <x:c r="B6" s="14" t="str">
+        <x:v>zbx-server-02</x:v>
+      </x:c>
+      <x:c r="C6" s="14" t="str">
+        <x:v>Zabbix Server standby</x:v>
+      </x:c>
+      <x:c r="D6" s="14" t="str">
+        <x:v>Producao</x:v>
+      </x:c>
+      <x:c r="E6" s="14" t="str"/>
+      <x:c r="F6" s="14" t="str"/>
+      <x:c r="G6" s="14" t="str"/>
+      <x:c r="H6" s="14" t="str"/>
+      <x:c r="I6" s="14" t="str"/>
+      <x:c r="J6" s="14" t="str">
+        <x:v>Nao</x:v>
+      </x:c>
+      <x:c r="K6" s="14" t="str"/>
+      <x:c r="L6" s="14" t="str">
+        <x:v>Pendente</x:v>
+      </x:c>
+      <x:c r="M6" s="14" t="str"/>
+    </x:row>
+    <x:row r="7" ht="15" hidden="0" customHeight="1">
+      <x:c r="A7" s="14" t="str">
+        <x:v>IP-003</x:v>
+      </x:c>
+      <x:c r="B7" s="14" t="str">
+        <x:v>zbx-fe-01</x:v>
+      </x:c>
+      <x:c r="C7" s="14" t="str">
+        <x:v>Frontend ativo</x:v>
+      </x:c>
+      <x:c r="D7" s="14" t="str">
+        <x:v>Producao</x:v>
+      </x:c>
+      <x:c r="E7" s="14" t="str"/>
+      <x:c r="F7" s="14" t="str"/>
+      <x:c r="G7" s="14" t="str"/>
+      <x:c r="H7" s="14" t="str"/>
+      <x:c r="I7" s="14" t="str"/>
+      <x:c r="J7" s="14" t="str">
+        <x:v>Nao</x:v>
+      </x:c>
+      <x:c r="K7" s="14" t="str"/>
+      <x:c r="L7" s="14" t="str">
+        <x:v>Pendente</x:v>
+      </x:c>
+      <x:c r="M7" s="14" t="str"/>
+    </x:row>
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
+      <x:c r="A8" s="14" t="str">
+        <x:v>IP-004</x:v>
+      </x:c>
+      <x:c r="B8" s="14" t="str">
+        <x:v>zbx-fe-02</x:v>
+      </x:c>
+      <x:c r="C8" s="14" t="str">
+        <x:v>Frontend standby</x:v>
+      </x:c>
+      <x:c r="D8" s="14" t="str">
+        <x:v>Producao</x:v>
+      </x:c>
+      <x:c r="E8" s="14" t="str"/>
+      <x:c r="F8" s="14" t="str"/>
+      <x:c r="G8" s="14" t="str"/>
+      <x:c r="H8" s="14" t="str"/>
+      <x:c r="I8" s="14" t="str"/>
+      <x:c r="J8" s="14" t="str">
+        <x:v>Nao</x:v>
+      </x:c>
+      <x:c r="K8" s="14" t="str"/>
+      <x:c r="L8" s="14" t="str">
+        <x:v>Pendente</x:v>
+      </x:c>
+      <x:c r="M8" s="14" t="str"/>
+    </x:row>
+    <x:row r="9" ht="15" hidden="0" customHeight="1">
+      <x:c r="A9" s="14" t="str">
+        <x:v>IP-005</x:v>
+      </x:c>
+      <x:c r="B9" s="14" t="str">
+        <x:v>pg-01</x:v>
+      </x:c>
+      <x:c r="C9" s="14" t="str">
+        <x:v>PostgreSQL Primary</x:v>
+      </x:c>
+      <x:c r="D9" s="14" t="str">
+        <x:v>Producao</x:v>
+      </x:c>
+      <x:c r="E9" s="14" t="str"/>
+      <x:c r="F9" s="14" t="str"/>
+      <x:c r="G9" s="14" t="str"/>
+      <x:c r="H9" s="14" t="str"/>
+      <x:c r="I9" s="14" t="str"/>
+      <x:c r="J9" s="14" t="str">
+        <x:v>Nao</x:v>
+      </x:c>
+      <x:c r="K9" s="14" t="str"/>
+      <x:c r="L9" s="14" t="str">
+        <x:v>Pendente</x:v>
+      </x:c>
+      <x:c r="M9" s="14" t="str">
+        <x:v>Banco deve ficar em rede de baixa latencia com Zabbix</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="15" hidden="0" customHeight="1">
+      <x:c r="A10" s="14" t="str">
+        <x:v>IP-006</x:v>
+      </x:c>
+      <x:c r="B10" s="14" t="str">
+        <x:v>pg-02</x:v>
+      </x:c>
+      <x:c r="C10" s="14" t="str">
+        <x:v>PostgreSQL Replica</x:v>
+      </x:c>
+      <x:c r="D10" s="14" t="str">
+        <x:v>Producao</x:v>
+      </x:c>
+      <x:c r="E10" s="14" t="str"/>
+      <x:c r="F10" s="14" t="str"/>
+      <x:c r="G10" s="14" t="str"/>
+      <x:c r="H10" s="14" t="str"/>
+      <x:c r="I10" s="14" t="str"/>
+      <x:c r="J10" s="14" t="str">
+        <x:v>Nao</x:v>
+      </x:c>
+      <x:c r="K10" s="14" t="str"/>
+      <x:c r="L10" s="14" t="str">
+        <x:v>Pendente</x:v>
+      </x:c>
+      <x:c r="M10" s="14" t="str">
+        <x:v>Mesmo segmento ou latencia adequada para replicacao</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="15" hidden="0" customHeight="1">
+      <x:c r="A11" s="14" t="str">
+        <x:v>IP-007</x:v>
+      </x:c>
+      <x:c r="B11" s="14" t="str">
+        <x:v>grafana-01</x:v>
+      </x:c>
+      <x:c r="C11" s="14" t="str">
+        <x:v>Grafana ativo</x:v>
+      </x:c>
+      <x:c r="D11" s="14" t="str">
+        <x:v>Producao</x:v>
+      </x:c>
+      <x:c r="E11" s="14" t="str"/>
+      <x:c r="F11" s="14" t="str"/>
+      <x:c r="G11" s="14" t="str"/>
+      <x:c r="H11" s="14" t="str"/>
+      <x:c r="I11" s="14" t="str"/>
+      <x:c r="J11" s="14" t="str">
+        <x:v>Condicional</x:v>
+      </x:c>
+      <x:c r="K11" s="14" t="str"/>
+      <x:c r="L11" s="14" t="str">
+        <x:v>Pendente</x:v>
+      </x:c>
+      <x:c r="M11" s="14" t="str"/>
+    </x:row>
+    <x:row r="12" ht="15" hidden="0" customHeight="1">
+      <x:c r="A12" s="14" t="str">
+        <x:v>IP-008</x:v>
+      </x:c>
+      <x:c r="B12" s="14" t="str">
+        <x:v>grafana-02</x:v>
+      </x:c>
+      <x:c r="C12" s="14" t="str">
+        <x:v>Grafana standby</x:v>
+      </x:c>
+      <x:c r="D12" s="14" t="str">
+        <x:v>Producao</x:v>
+      </x:c>
+      <x:c r="E12" s="14" t="str"/>
+      <x:c r="F12" s="14" t="str"/>
+      <x:c r="G12" s="14" t="str"/>
+      <x:c r="H12" s="14" t="str"/>
+      <x:c r="I12" s="14" t="str"/>
+      <x:c r="J12" s="14" t="str">
+        <x:v>Condicional</x:v>
+      </x:c>
+      <x:c r="K12" s="14" t="str"/>
+      <x:c r="L12" s="14" t="str">
+        <x:v>Pendente</x:v>
+      </x:c>
+      <x:c r="M12" s="14" t="str"/>
+    </x:row>
+    <x:row r="13" ht="15" hidden="0" customHeight="1">
+      <x:c r="A13" s="14" t="str">
+        <x:v>IP-009</x:v>
+      </x:c>
+      <x:c r="B13" s="14" t="str">
+        <x:v>awx-01</x:v>
+      </x:c>
+      <x:c r="C13" s="14" t="str">
+        <x:v>AWX ativo</x:v>
+      </x:c>
+      <x:c r="D13" s="14" t="str">
+        <x:v>Producao</x:v>
+      </x:c>
+      <x:c r="E13" s="14" t="str"/>
+      <x:c r="F13" s="14" t="str"/>
+      <x:c r="G13" s="14" t="str"/>
+      <x:c r="H13" s="14" t="str"/>
+      <x:c r="I13" s="14" t="str"/>
+      <x:c r="J13" s="14" t="str">
+        <x:v>Condicional</x:v>
+      </x:c>
+      <x:c r="K13" s="14" t="str"/>
+      <x:c r="L13" s="14" t="str">
+        <x:v>Pendente</x:v>
+      </x:c>
+      <x:c r="M13" s="14" t="str"/>
+    </x:row>
+    <x:row r="14" ht="15" hidden="0" customHeight="1">
+      <x:c r="A14" s="14" t="str">
+        <x:v>IP-010</x:v>
+      </x:c>
+      <x:c r="B14" s="14" t="str">
+        <x:v>awx-02</x:v>
+      </x:c>
+      <x:c r="C14" s="14" t="str">
+        <x:v>AWX standby opcional</x:v>
+      </x:c>
+      <x:c r="D14" s="14" t="str">
+        <x:v>Producao</x:v>
+      </x:c>
+      <x:c r="E14" s="14" t="str"/>
+      <x:c r="F14" s="14" t="str"/>
+      <x:c r="G14" s="14" t="str"/>
+      <x:c r="H14" s="14" t="str"/>
+      <x:c r="I14" s="14" t="str"/>
+      <x:c r="J14" s="14" t="str">
+        <x:v>Condicional</x:v>
+      </x:c>
+      <x:c r="K14" s="14" t="str"/>
+      <x:c r="L14" s="14" t="str">
+        <x:v>Pendente</x:v>
+      </x:c>
+      <x:c r="M14" s="14" t="str">
+        <x:v>Preencher se AWX standby for aprovado</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="15" hidden="0" customHeight="1">
+      <x:c r="A15" s="14" t="str">
+        <x:v>IP-011</x:v>
+      </x:c>
+      <x:c r="B15" s="14" t="str">
+        <x:v>vip-01</x:v>
+      </x:c>
+      <x:c r="C15" s="14" t="str">
+        <x:v>Keepalived + Proxy ativo</x:v>
+      </x:c>
+      <x:c r="D15" s="14" t="str">
+        <x:v>Producao</x:v>
+      </x:c>
+      <x:c r="E15" s="14" t="str"/>
+      <x:c r="F15" s="14" t="str"/>
+      <x:c r="G15" s="14" t="str"/>
+      <x:c r="H15" s="14" t="str"/>
+      <x:c r="I15" s="14" t="str"/>
+      <x:c r="J15" s="14" t="str">
+        <x:v>Condicional</x:v>
+      </x:c>
+      <x:c r="K15" s="14" t="str"/>
+      <x:c r="L15" s="14" t="str">
+        <x:v>Pendente</x:v>
+      </x:c>
+      <x:c r="M15" s="14" t="str"/>
+    </x:row>
+    <x:row r="16" ht="15" hidden="0" customHeight="1">
+      <x:c r="A16" s="14" t="str">
+        <x:v>IP-012</x:v>
+      </x:c>
+      <x:c r="B16" s="14" t="str">
+        <x:v>vip-02</x:v>
+      </x:c>
+      <x:c r="C16" s="14" t="str">
+        <x:v>Keepalived + Proxy standby</x:v>
+      </x:c>
+      <x:c r="D16" s="14" t="str">
+        <x:v>Producao</x:v>
+      </x:c>
+      <x:c r="E16" s="14" t="str"/>
+      <x:c r="F16" s="14" t="str"/>
+      <x:c r="G16" s="14" t="str"/>
+      <x:c r="H16" s="14" t="str"/>
+      <x:c r="I16" s="14" t="str"/>
+      <x:c r="J16" s="14" t="str">
+        <x:v>Condicional</x:v>
+      </x:c>
+      <x:c r="K16" s="14" t="str"/>
+      <x:c r="L16" s="14" t="str">
+        <x:v>Pendente</x:v>
+      </x:c>
+      <x:c r="M16" s="14" t="str"/>
+    </x:row>
+    <x:row r="17" ht="15" hidden="0" customHeight="1">
+      <x:c r="A17" s="14" t="str">
+        <x:v>IP-013</x:v>
+      </x:c>
+      <x:c r="B17" s="14" t="str">
+        <x:v>VIP-Zabbix-Web</x:v>
+      </x:c>
+      <x:c r="C17" s="14" t="str">
+        <x:v>VIP acesso Zabbix Frontend</x:v>
+      </x:c>
+      <x:c r="D17" s="14" t="str">
+        <x:v>Producao</x:v>
+      </x:c>
+      <x:c r="E17" s="14" t="str"/>
+      <x:c r="F17" s="14" t="str"/>
+      <x:c r="G17" s="14" t="str"/>
+      <x:c r="H17" s="14" t="str"/>
+      <x:c r="I17" s="14" t="str"/>
+      <x:c r="J17" s="14" t="str">
+        <x:v>Condicional</x:v>
+      </x:c>
+      <x:c r="K17" s="14" t="str"/>
+      <x:c r="L17" s="14" t="str">
+        <x:v>Pendente</x:v>
+      </x:c>
+      <x:c r="M17" s="14" t="str">
+        <x:v>Nome DNS recomendado</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="15" hidden="0" customHeight="1">
+      <x:c r="A18" s="14" t="str">
+        <x:v>IP-014</x:v>
+      </x:c>
+      <x:c r="B18" s="14" t="str">
+        <x:v>VIP-Grafana</x:v>
+      </x:c>
+      <x:c r="C18" s="14" t="str">
+        <x:v>VIP acesso Grafana</x:v>
+      </x:c>
+      <x:c r="D18" s="14" t="str">
+        <x:v>Producao</x:v>
+      </x:c>
+      <x:c r="E18" s="14" t="str"/>
+      <x:c r="F18" s="14" t="str"/>
+      <x:c r="G18" s="14" t="str"/>
+      <x:c r="H18" s="14" t="str"/>
+      <x:c r="I18" s="14" t="str"/>
+      <x:c r="J18" s="14" t="str">
+        <x:v>Condicional</x:v>
+      </x:c>
+      <x:c r="K18" s="14" t="str"/>
+      <x:c r="L18" s="14" t="str">
+        <x:v>Pendente</x:v>
+      </x:c>
+      <x:c r="M18" s="14" t="str">
+        <x:v>Pode compartilhar proxy/VIP conforme desenho aprovado</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="15" hidden="0" customHeight="1">
+      <x:c r="A19" s="14" t="str">
+        <x:v>IP-015</x:v>
+      </x:c>
+      <x:c r="B19" s="14" t="str">
+        <x:v>VIP-AWX</x:v>
+      </x:c>
+      <x:c r="C19" s="14" t="str">
+        <x:v>VIP acesso AWX</x:v>
+      </x:c>
+      <x:c r="D19" s="14" t="str">
+        <x:v>Producao</x:v>
+      </x:c>
+      <x:c r="E19" s="14" t="str"/>
+      <x:c r="F19" s="14" t="str"/>
+      <x:c r="G19" s="14" t="str"/>
+      <x:c r="H19" s="14" t="str"/>
+      <x:c r="I19" s="14" t="str"/>
+      <x:c r="J19" s="14" t="str">
+        <x:v>Condicional</x:v>
+      </x:c>
+      <x:c r="K19" s="14" t="str"/>
+      <x:c r="L19" s="14" t="str">
+        <x:v>Pendente</x:v>
+      </x:c>
+      <x:c r="M19" s="14" t="str">
+        <x:v>Pode compartilhar proxy/VIP conforme desenho aprovado</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:M1"/>
+    <x:mergeCell ref="A2:H2"/>
+  </x:mergeCells>
+  <x:conditionalFormatting sqref="L5:L40">
+    <x:cfRule type="containsText" dxfId="20" priority="1" operator="containsText" text="Concluido"/>
+    <x:cfRule type="containsText" dxfId="21" priority="2" operator="containsText" text="Em andamento"/>
+    <x:cfRule type="containsText" dxfId="22" priority="3" operator="containsText" text="Pendente"/>
+    <x:cfRule type="containsText" dxfId="23" priority="4" operator="containsText" text="Nao aplicavel"/>
+  </x:conditionalFormatting>
+  <x:dataValidations count="2">
+    <x:dataValidation type="list" sqref="J5:J40">
+      <x:formula1>"Sim,Nao,Condicional"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="L5:L40">
+      <x:formula1>"Pendente,Em andamento,Concluido,Nao aplicavel"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
     <x:col min="1" max="1" width="50" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="27.5" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="27.5" hidden="0" customWidth="1"/>
@@ -17273,10 +18148,10 @@
     <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="H5:H40">
-    <x:cfRule type="containsText" dxfId="20" priority="1" operator="containsText" text="Concluido"/>
-    <x:cfRule type="containsText" dxfId="21" priority="2" operator="containsText" text="Em andamento"/>
-    <x:cfRule type="containsText" dxfId="22" priority="3" operator="containsText" text="Pendente"/>
-    <x:cfRule type="containsText" dxfId="23" priority="4" operator="containsText" text="Nao aplicavel"/>
+    <x:cfRule type="containsText" dxfId="24" priority="1" operator="containsText" text="Concluido"/>
+    <x:cfRule type="containsText" dxfId="25" priority="2" operator="containsText" text="Em andamento"/>
+    <x:cfRule type="containsText" dxfId="26" priority="3" operator="containsText" text="Pendente"/>
+    <x:cfRule type="containsText" dxfId="27" priority="4" operator="containsText" text="Nao aplicavel"/>
   </x:conditionalFormatting>
   <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="F5:F40">
@@ -17290,7 +18165,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -17576,10 +18451,10 @@
     <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="H5:H40">
-    <x:cfRule type="containsText" dxfId="24" priority="1" operator="containsText" text="Concluido"/>
-    <x:cfRule type="containsText" dxfId="25" priority="2" operator="containsText" text="Em andamento"/>
-    <x:cfRule type="containsText" dxfId="26" priority="3" operator="containsText" text="Pendente"/>
-    <x:cfRule type="containsText" dxfId="27" priority="4" operator="containsText" text="Nao aplicavel"/>
+    <x:cfRule type="containsText" dxfId="28" priority="1" operator="containsText" text="Concluido"/>
+    <x:cfRule type="containsText" dxfId="29" priority="2" operator="containsText" text="Em andamento"/>
+    <x:cfRule type="containsText" dxfId="30" priority="3" operator="containsText" text="Pendente"/>
+    <x:cfRule type="containsText" dxfId="31" priority="4" operator="containsText" text="Nao aplicavel"/>
   </x:conditionalFormatting>
   <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="G5:G40">
@@ -17593,7 +18468,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -17887,10 +18762,10 @@
     <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="H5:H30">
-    <x:cfRule type="containsText" dxfId="28" priority="1" operator="containsText" text="Concluido"/>
-    <x:cfRule type="containsText" dxfId="29" priority="2" operator="containsText" text="Em andamento"/>
-    <x:cfRule type="containsText" dxfId="30" priority="3" operator="containsText" text="Pendente"/>
-    <x:cfRule type="containsText" dxfId="31" priority="4" operator="containsText" text="Nao aplicavel"/>
+    <x:cfRule type="containsText" dxfId="32" priority="1" operator="containsText" text="Concluido"/>
+    <x:cfRule type="containsText" dxfId="33" priority="2" operator="containsText" text="Em andamento"/>
+    <x:cfRule type="containsText" dxfId="34" priority="3" operator="containsText" text="Pendente"/>
+    <x:cfRule type="containsText" dxfId="35" priority="4" operator="containsText" text="Nao aplicavel"/>
   </x:conditionalFormatting>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="H5:H30">
@@ -17899,204 +18774,4 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="52.380001068115234" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="52.380001068115234" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="52.380001068115234" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="52.380001068115234" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="52.380001068115234" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="31.25" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="31.25" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="31.25" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" ht="19.200000762939453" hidden="0" customHeight="1">
-      <x:c r="A1" s="6" t="str">
-        <x:v>Contatos e Responsaveis</x:v>
-      </x:c>
-      <x:c r="B1" s="6" t="str">
-        <x:v>Contatos e Responsaveis</x:v>
-      </x:c>
-      <x:c r="C1" s="6" t="str">
-        <x:v>Contatos e Responsaveis</x:v>
-      </x:c>
-      <x:c r="D1" s="6" t="str">
-        <x:v>Contatos e Responsaveis</x:v>
-      </x:c>
-      <x:c r="E1" s="6" t="str">
-        <x:v>Contatos e Responsaveis</x:v>
-      </x:c>
-      <x:c r="F1" s="6" t="str">
-        <x:v>Contatos e Responsaveis</x:v>
-      </x:c>
-      <x:c r="G1" s="6" t="str">
-        <x:v>Contatos e Responsaveis</x:v>
-      </x:c>
-      <x:c r="H1" s="6" t="str">
-        <x:v>Contatos e Responsaveis</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" ht="15" hidden="0" customHeight="1">
-      <x:c r="A2" s="11" t="str">
-        <x:v>Preencher responsaveis por area para aprovacoes, duvidas e escalonamento.</x:v>
-      </x:c>
-      <x:c r="B2" s="11" t="str">
-        <x:v>Preencher responsaveis por area para aprovacoes, duvidas e escalonamento.</x:v>
-      </x:c>
-      <x:c r="C2" s="11" t="str">
-        <x:v>Preencher responsaveis por area para aprovacoes, duvidas e escalonamento.</x:v>
-      </x:c>
-      <x:c r="D2" s="11" t="str">
-        <x:v>Preencher responsaveis por area para aprovacoes, duvidas e escalonamento.</x:v>
-      </x:c>
-      <x:c r="E2" s="11" t="str">
-        <x:v>Preencher responsaveis por area para aprovacoes, duvidas e escalonamento.</x:v>
-      </x:c>
-      <x:c r="F2" s="11" t="str">
-        <x:v>Preencher responsaveis por area para aprovacoes, duvidas e escalonamento.</x:v>
-      </x:c>
-      <x:c r="G2" s="11" t="str">
-        <x:v>Preencher responsaveis por area para aprovacoes, duvidas e escalonamento.</x:v>
-      </x:c>
-      <x:c r="H2" s="11" t="str">
-        <x:v>Preencher responsaveis por area para aprovacoes, duvidas e escalonamento.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3"/>
-    <x:row r="4" ht="15" hidden="0" customHeight="1">
-      <x:c r="A4" s="17" t="str">
-        <x:v>Area</x:v>
-      </x:c>
-      <x:c r="B4" s="17" t="str">
-        <x:v>Nome</x:v>
-      </x:c>
-      <x:c r="C4" s="17" t="str">
-        <x:v>Cargo/Funcao</x:v>
-      </x:c>
-      <x:c r="D4" s="17" t="str">
-        <x:v>E-mail</x:v>
-      </x:c>
-      <x:c r="E4" s="17" t="str">
-        <x:v>Telefone</x:v>
-      </x:c>
-      <x:c r="F4" s="17" t="str">
-        <x:v>Responsabilidade</x:v>
-      </x:c>
-      <x:c r="G4" s="17" t="str">
-        <x:v>Backup</x:v>
-      </x:c>
-      <x:c r="H4" s="17" t="str">
-        <x:v>Observacoes</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="15" hidden="0" customHeight="1">
-      <x:c r="A5" s="14" t="str">
-        <x:v>Gestao do projeto</x:v>
-      </x:c>
-      <x:c r="B5" s="14" t="str"/>
-      <x:c r="C5" s="14" t="str"/>
-      <x:c r="D5" s="14" t="str"/>
-      <x:c r="E5" s="14" t="str"/>
-      <x:c r="F5" s="14" t="str">
-        <x:v>Aprovacao de cronograma e status report</x:v>
-      </x:c>
-      <x:c r="G5" s="14" t="str"/>
-      <x:c r="H5" s="14" t="str"/>
-    </x:row>
-    <x:row r="6" ht="15" hidden="0" customHeight="1">
-      <x:c r="A6" s="14" t="str">
-        <x:v>Rede</x:v>
-      </x:c>
-      <x:c r="B6" s="14" t="str"/>
-      <x:c r="C6" s="14" t="str"/>
-      <x:c r="D6" s="14" t="str"/>
-      <x:c r="E6" s="14" t="str"/>
-      <x:c r="F6" s="14" t="str">
-        <x:v>Portas, VLANs, ACLs, QoS e roteamento</x:v>
-      </x:c>
-      <x:c r="G6" s="14" t="str"/>
-      <x:c r="H6" s="14" t="str"/>
-    </x:row>
-    <x:row r="7" ht="15" hidden="0" customHeight="1">
-      <x:c r="A7" s="14" t="str">
-        <x:v>Seguranca</x:v>
-      </x:c>
-      <x:c r="B7" s="14" t="str"/>
-      <x:c r="C7" s="14" t="str"/>
-      <x:c r="D7" s="14" t="str"/>
-      <x:c r="E7" s="14" t="str"/>
-      <x:c r="F7" s="14" t="str">
-        <x:v>VPN, credenciais, certificados e RBAC</x:v>
-      </x:c>
-      <x:c r="G7" s="14" t="str"/>
-      <x:c r="H7" s="14" t="str"/>
-    </x:row>
-    <x:row r="8" ht="15" hidden="0" customHeight="1">
-      <x:c r="A8" s="14" t="str">
-        <x:v>Infraestrutura</x:v>
-      </x:c>
-      <x:c r="B8" s="14" t="str"/>
-      <x:c r="C8" s="14" t="str"/>
-      <x:c r="D8" s="14" t="str"/>
-      <x:c r="E8" s="14" t="str"/>
-      <x:c r="F8" s="14" t="str">
-        <x:v>VMs, storage, DNS, NTP e SO</x:v>
-      </x:c>
-      <x:c r="G8" s="14" t="str"/>
-      <x:c r="H8" s="14" t="str"/>
-    </x:row>
-    <x:row r="9" ht="15" hidden="0" customHeight="1">
-      <x:c r="A9" s="14" t="str">
-        <x:v>Banco de dados</x:v>
-      </x:c>
-      <x:c r="B9" s="14" t="str"/>
-      <x:c r="C9" s="14" t="str"/>
-      <x:c r="D9" s="14" t="str"/>
-      <x:c r="E9" s="14" t="str"/>
-      <x:c r="F9" s="14" t="str">
-        <x:v>PostgreSQL, backup, restore e performance</x:v>
-      </x:c>
-      <x:c r="G9" s="14" t="str"/>
-      <x:c r="H9" s="14" t="str"/>
-    </x:row>
-    <x:row r="10" ht="15" hidden="0" customHeight="1">
-      <x:c r="A10" s="14" t="str">
-        <x:v>Operacao/NOC</x:v>
-      </x:c>
-      <x:c r="B10" s="14" t="str"/>
-      <x:c r="C10" s="14" t="str"/>
-      <x:c r="D10" s="14" t="str"/>
-      <x:c r="E10" s="14" t="str"/>
-      <x:c r="F10" s="14" t="str">
-        <x:v>Recebimento de alertas e operacao assistida</x:v>
-      </x:c>
-      <x:c r="G10" s="14" t="str"/>
-      <x:c r="H10" s="14" t="str"/>
-    </x:row>
-    <x:row r="11" ht="15" hidden="0" customHeight="1">
-      <x:c r="A11" s="14" t="str">
-        <x:v>Aplicacoes</x:v>
-      </x:c>
-      <x:c r="B11" s="14" t="str"/>
-      <x:c r="C11" s="14" t="str"/>
-      <x:c r="D11" s="14" t="str"/>
-      <x:c r="E11" s="14" t="str"/>
-      <x:c r="F11" s="14" t="str">
-        <x:v>Validacao de servicos monitorados</x:v>
-      </x:c>
-      <x:c r="G11" s="14" t="str"/>
-      <x:c r="H11" s="14" t="str"/>
-    </x:row>
-  </x:sheetData>
-  <x:mergeCells>
-    <x:mergeCell ref="A1:H1"/>
-    <x:mergeCell ref="A2:H2"/>
-  </x:mergeCells>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</x:worksheet>
 </file>
</xml_diff>